<commit_message>
Dashboard 2026-09-10 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/339853872/spec-339853872.xlsx
+++ b/vse-loti/339853872/spec-339853872.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0.0000"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00&quot; ₽&quot;"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00&quot; ₽&quot;"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -83,17 +82,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -462,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -529,7 +526,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Труба стальная бесшовная предизолированная 273×7/400 ППУ-ПЭ (сталь 20 ГОСТ 8732-78, изоляция ГОСТ 30732-2006) М.п. 432 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт качества, сертификат соответствия, транспортные документы, инструкция по эксплуатации 2. Отвод стальной крутоизогнутый 90° ППУ Ду250 (273*7 мм) ГОСТ 17375 Шт. 14 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт, транспортные документы, сертификат соответствия инструкция по эксплуатации 3. Отвод стальной 45° ППУ Ду250 ГОСТ 17375</t>
+          <t>Труба стальная бесшовная предизолированная 273×7/400 ППУ-ПЭ (сталь 20 ГОСТ 8732-78, изоляция ГОСТ 30732-2006)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -538,11 +535,11 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2001</v>
+        <v>432</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>М.п.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -555,16 +552,16 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Комплект для заделки стыков труб ППУ ГОСТ 30732</t>
+          <t>Отвод стальнойкрутоизогнутый 90° ППУДу250 (273*7 мм) ГОСТ 17375</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" s="3" t="n">
-        <v>2020</v>
+        <v>14</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>Шт.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -577,16 +574,16 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Комплект фланцевый Ду250 PN16 (фланцы, крепёж, прокладки) ГОСТ 33259-2015, ГОСТ 7798-70, ГОСТ 9066-75, ГОСТ 15180</t>
+          <t>Отвод стальной 45° ППУДу250 ГОСТ 17375-2001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" s="3" t="n">
-        <v>86</v>
+        <v>2</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>Шт.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -599,25 +596,19 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Труба стальная цельнокатаная (бесшовная) 219×6 ГОСТ 8732</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>219×6</t>
-        </is>
-      </c>
+          <t>Комплект для заделкистыков труб ППУ ГОСТ 30732-2020</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" s="3" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>м</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>2.459</v>
-      </c>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -627,25 +618,19 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Труба стальная цельнокатаная (бесшовная) 89×5 ГОСТ 8732</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>89×5</t>
-        </is>
-      </c>
+          <t>Кран шаровый фланцевыйДу250 PN16 ст.20(полнопроходной) ГОСТ21345-2005, ГОСТ 12815-80</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" s="3" t="n">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>м</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>0.8080000000000001</v>
-      </c>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -655,16 +640,16 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Комплект фланцевый Ду80 PN16 (фланцы, крепёж, прокладки) ГОСТ 33259</t>
+          <t>Комплект фланцевый Ду250PN16 (фланцы, крепёж,прокладки) ГОСТ 33259-2015,ГОСТ 7798-70, ГОСТ 9066-75,ГОСТ 15180-86</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" s="3" t="n">
-        <v>2015</v>
+        <v>2</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>Шт.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -677,16 +662,16 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Комплект фланцевый Ду200 PN16 (фланцы, крепёж, прокладки) ГОСТ 33259</t>
+          <t>Шаровый кран ГОСТ, PN40, Ду 50, ВР 2" рычаг 8756</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" s="3" t="n">
-        <v>2015</v>
+        <v>2</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>Шт.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -699,25 +684,19 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Труба стальная бесшовная предизолированная 273×7/400 ППУ-ПЭ (сталь 20 ГОСТ 8732-78, изоляция ГОСТ 30732-2006) М.п. 432 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт качества, сертификат соответствия, транспортные документы, инструкция по эксплуатации 2. Отвод стальной крутоизогнутый 90° ППУ Ду250 (273*7 мм) ГОСТ 17375 Шт. 14 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт, транспортные документы, сертификат соответствия инструкция по эксплуатации 3. Отвод стальной 45° ППУ Ду250 ГОСТ 17375-2001 Шт. 2 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт, транспортные документы, сертификат соответствия, инструкция по эксплуатации 4. Комплект для заделки стыков труб ППУ ГОСТ 30732- 2020 Шт. 70 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт, транспортные документы, сертификат соответствия, инструкция по эксплуатации 5. Кран шаровый фланцевый Ду250 PN16 ст.20 (полнопроходной) ГОСТ 21345-2005, ГОСТ 12815-80 Шт. 2 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт, транспортные документы, сертификат соответствия, инструкция по эксплуатации 6. Комплект фланцевый Ду250 PN16 (фланцы, крепёж, прокладки) ГОСТ 33259-2015, ГОСТ 7798-70, ГОСТ 9066-75, ГОСТ 15180-86 Шт. 2 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт, транспортные документы, сертификат соответствия, инструкция по эксплуатации 7. Шаровый кран ГОСТ, PN40, Ду 50, ВР 2" рычаг 8756 Шт. 2 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт, транспортные документы, сертификат соответствия, инструкция по эксплуатации 8. Шаровый кран ГОСТ, PN40, Ду 32, ВР 1 1/4" рычаг 8754 Шт. 2 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт, транспортные документы, сертификат соответствия, инструкция по эксплуатации 9. Переход стальной исп 2 концентр Дн273х219-7х6 (Ду250х200) б/шовный ГОСТ 17378-2001 Шт. 4 30 календарных дней Нижегородская обл, Нижний Новгород г, Баррикад ул, д. 1. Паспорт, транспортные документы, сертификат соответствия, инструкция по эксплуатации 10. Труба стальная цельнокатаная (бесшовная) 219×6 ГОСТ 8732-</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>273×7</t>
-        </is>
-      </c>
+          <t>Шаровый кран ГОСТ, PN40, Ду 32, ВР 1 1/4" рычаг 8754</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" s="3" t="n">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>м</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>0.433</v>
-      </c>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -727,61 +706,262 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Труба стальная цельнокатаная (бесшовная) 89×5 ГОСТ 8732-7</t>
+          <t>Переход стальной исп 2 концентр Дн273х219-7х6 (Ду250х200) б/шовный ГОСТ 17378-2001</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>89×5</t>
+          <t>273×219</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>м</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>0.083</v>
-      </c>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Труба стальная цельнокатаная (бесшовная) 219×6 ГОСТ 8732-78</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>219×6</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>М.п.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Отвод стальной крутоизогнутый 90° Ду200 ГОСТ 17375-2001</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Труба стальная цельнокатаная (бесшовная) 89×5 ГОСТ 8732-78</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>89×5</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>М.п.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Отвод стальной крутоизогнутый 90° Ду80 ГОСТ 17375-2001</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Кран шаровый фланцевыйДу80 PN16 ст.20(полнопроходной) ГОСТ21345-2005, ГОСТ 12815-80</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Комплект фланцевый Ду80PN16 (фланцы, крепёж,прокладки) ГОСТ 33259-2015</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Комплект фланцевый Ду200PN16 (фланцы, крепёж,прокладки) ГОСТ 33259-2015</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Плита перекрытия лотка П 15-8/2 1495*1840*120</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Лоток теплотрасс Л 11-8</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Шт.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
-        <v>3.783</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>НМЦК из обоснования:</t>
         </is>
       </c>
-      <c r="G12" s="7" t="n">
+      <c r="G21" s="5" t="n">
         <v>12560000</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Источник: Документация 11.08.2026.docx
 Приложение № 2. Техническое задание.docx</t>
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
+    <row r="24"/>
+    <row r="25"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A14:B16"/>
+    <mergeCell ref="A23:B25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>